<commit_message>
UI: amélioration page d'accueil + design system cartes
</commit_message>
<xml_diff>
--- a/Donnees/Pauvreté et condition de vie/Conditions de vie/Theme_Conditions_de_vie.xlsx
+++ b/Donnees/Pauvreté et condition de vie/Conditions de vie/Theme_Conditions_de_vie.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Documents\Ansade_Project\Donnees\Pauvreté et condition de vie\Conditions de vie\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87C64B0F-1C1F-469A-919F-9115E0DFCF4C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F377E0B4-5EE7-423E-9F09-402AD096A170}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="st_occuplog" sheetId="1" r:id="rId1"/>
@@ -26,9 +26,6 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="28">
   <si>
-    <t>Tableau 2.2.1: Proportion(%) de ménages propriétaire du logement occupé (avec ou sans titre de propriété)</t>
-  </si>
-  <si>
     <t>2004</t>
   </si>
   <si>
@@ -95,19 +92,22 @@
     <t>Source : EPCV/2004-2019</t>
   </si>
   <si>
-    <t>Tableau 2.2.2: Proportion(%) de ménages disposant de robinet pour l'approvisionnement en eau de boisson</t>
-  </si>
-  <si>
-    <t>Tableau 2.2.3: Proportion(%) de ménages s'approvisionnent en eau de boisson à partir de source améliorée (robinet, forage, borne fontaine, puits protégé)</t>
-  </si>
-  <si>
-    <t>Tableau 2.2.4: Proportion de ménages ne possédant pas de toilette</t>
-  </si>
-  <si>
-    <t>Tableau 2.2.5: Proportion de ménages utilisant des énergies propres pour la cuisson (gaz, électricité)</t>
-  </si>
-  <si>
     <t>Total</t>
+  </si>
+  <si>
+    <t>Tableau 2.2.1: Proportion (%) de ménages propriétaires du logement occupé (avec ou sans titre de propriété)</t>
+  </si>
+  <si>
+    <t>Tableau 2.2.2: Proportion (%) de ménages disposant de robinet pour l'approvisionnement en eau de boisson</t>
+  </si>
+  <si>
+    <t>Tableau 2.2.3: Proportion (%) de ménages s'approvisionnant en eau de boisson à partir de sources améliorées (robinet, forage, borne fontaine, puits protégé)</t>
+  </si>
+  <si>
+    <t>Tableau 2.2.4: Proportion (%) de ménages ne possédant pas de toilette</t>
+  </si>
+  <si>
+    <t>Tableau 2.2.5: Proportion (%) de ménages utilisant des énergies propres pour la cuisson (gaz, électricité)</t>
   </si>
 </sst>
 </file>
@@ -473,27 +473,27 @@
   <sheetData>
     <row r="1" spans="1:5" ht="17.399999999999999" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>0</v>
+        <v>23</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" s="2"/>
       <c r="B2" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="D2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="E2" s="2" t="s">
         <v>3</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="B3">
         <v>0.80220000000000002</v>
@@ -510,7 +510,7 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B4">
         <v>0.58309999999999995</v>
@@ -527,7 +527,7 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B5">
         <v>0.94120000000000004</v>
@@ -544,7 +544,7 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B6">
         <v>0.96220000000000006</v>
@@ -561,7 +561,7 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B7">
         <v>0.92459999999999998</v>
@@ -578,7 +578,7 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B8">
         <v>0.95469999999999999</v>
@@ -595,7 +595,7 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B9">
         <v>0.94640000000000002</v>
@@ -612,7 +612,7 @@
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B10">
         <v>0.89659999999999995</v>
@@ -629,7 +629,7 @@
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B11">
         <v>0.90639999999999998</v>
@@ -646,7 +646,7 @@
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B12">
         <v>0.61719999999999997</v>
@@ -663,7 +663,7 @@
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B13">
         <v>0.47210000000000002</v>
@@ -680,7 +680,7 @@
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B14">
         <v>0.6956</v>
@@ -697,7 +697,7 @@
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B15">
         <v>0.94340000000000002</v>
@@ -714,7 +714,7 @@
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B16">
         <v>0.52300000000000002</v>
@@ -731,7 +731,7 @@
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B17">
         <v>0.64090000000000003</v>
@@ -748,7 +748,7 @@
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B18">
         <v>0.45100000000000001</v>
@@ -765,7 +765,7 @@
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B19">
         <v>0.80169999999999997</v>
@@ -782,7 +782,7 @@
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B20">
         <v>0.80410000000000004</v>
@@ -799,7 +799,7 @@
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A24" s="3" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
   </sheetData>
@@ -811,30 +811,33 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:E23"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="113.88671875" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="17.399999999999999" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" s="2"/>
       <c r="B2" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="D2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="E2" s="2" t="s">
         <v>3</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="B3">
         <v>0.26910000000000001</v>
@@ -851,7 +854,7 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B4">
         <v>0.4249</v>
@@ -868,7 +871,7 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B5">
         <v>0.17030000000000001</v>
@@ -885,7 +888,7 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B6">
         <v>0.159</v>
@@ -902,7 +905,7 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B7">
         <v>0.2361</v>
@@ -919,7 +922,7 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B8">
         <v>0.1991</v>
@@ -936,7 +939,7 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B9">
         <v>0.1744</v>
@@ -953,7 +956,7 @@
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B10">
         <v>0.2228</v>
@@ -970,7 +973,7 @@
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B11">
         <v>0.53859999999999997</v>
@@ -987,7 +990,7 @@
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B12">
         <v>0.2069</v>
@@ -1004,7 +1007,7 @@
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B13">
         <v>0.4889</v>
@@ -1021,7 +1024,7 @@
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B14">
         <v>0.223</v>
@@ -1038,7 +1041,7 @@
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B15">
         <v>9.3100000000000002E-2</v>
@@ -1055,7 +1058,7 @@
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B16">
         <v>0.46550000000000002</v>
@@ -1072,7 +1075,7 @@
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B17">
         <v>0.69489999999999996</v>
@@ -1089,7 +1092,7 @@
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B18">
         <v>0.30940000000000001</v>
@@ -1106,7 +1109,7 @@
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B19">
         <v>0.26219999999999999</v>
@@ -1123,7 +1126,7 @@
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B20">
         <v>0.29830000000000001</v>
@@ -1140,7 +1143,7 @@
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A23" s="3" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
   </sheetData>
@@ -1155,27 +1158,27 @@
   <sheetData>
     <row r="1" spans="1:5" ht="17.399999999999999" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" s="2"/>
       <c r="B2" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="D2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="E2" s="2" t="s">
         <v>3</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="B3">
         <v>0.32069999999999999</v>
@@ -1192,7 +1195,7 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B4">
         <v>0.42730000000000001</v>
@@ -1209,7 +1212,7 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B5">
         <v>0.25309999999999999</v>
@@ -1226,7 +1229,7 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B6">
         <v>0.2054</v>
@@ -1243,7 +1246,7 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B7">
         <v>0.26090000000000002</v>
@@ -1260,7 +1263,7 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B8">
         <v>0.30780000000000002</v>
@@ -1277,7 +1280,7 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B9">
         <v>0.2611</v>
@@ -1294,7 +1297,7 @@
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B10">
         <v>0.27689999999999998</v>
@@ -1311,7 +1314,7 @@
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B11">
         <v>0.59609999999999996</v>
@@ -1328,7 +1331,7 @@
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B12">
         <v>0.29380000000000001</v>
@@ -1345,7 +1348,7 @@
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B13">
         <v>0.49380000000000002</v>
@@ -1362,7 +1365,7 @@
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B14">
         <v>0.30380000000000001</v>
@@ -1379,7 +1382,7 @@
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B15">
         <v>0.18840000000000001</v>
@@ -1396,7 +1399,7 @@
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B16">
         <v>0.46550000000000002</v>
@@ -1413,7 +1416,7 @@
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B17">
         <v>0.71379999999999999</v>
@@ -1430,7 +1433,7 @@
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B18">
         <v>0.30940000000000001</v>
@@ -1447,7 +1450,7 @@
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B19">
         <v>0.42730000000000001</v>
@@ -1464,7 +1467,7 @@
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B20">
         <v>0.25309999999999999</v>
@@ -1481,7 +1484,7 @@
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A23" s="3" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
   </sheetData>
@@ -1499,27 +1502,27 @@
   <sheetData>
     <row r="1" spans="1:5" ht="17.399999999999999" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" s="2"/>
       <c r="B2" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="D2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="E2" s="2" t="s">
         <v>3</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="B3">
         <v>0.51029999999999998</v>
@@ -1536,7 +1539,7 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B4">
         <v>0.1857</v>
@@ -1553,7 +1556,7 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B5">
         <v>0.71630000000000005</v>
@@ -1570,7 +1573,7 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B6">
         <v>0.59219999999999995</v>
@@ -1587,7 +1590,7 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B7">
         <v>0.77649999999999997</v>
@@ -1604,7 +1607,7 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B8">
         <v>0.75019999999999998</v>
@@ -1621,7 +1624,7 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B9">
         <v>0.65690000000000004</v>
@@ -1638,7 +1641,7 @@
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B10">
         <v>0.61370000000000002</v>
@@ -1655,7 +1658,7 @@
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B11">
         <v>0.59560000000000002</v>
@@ -1672,7 +1675,7 @@
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B12">
         <v>0.45910000000000001</v>
@@ -1689,7 +1692,7 @@
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B13">
         <v>0.17599999999999999</v>
@@ -1706,7 +1709,7 @@
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B14">
         <v>0.79069999999999996</v>
@@ -1723,7 +1726,7 @@
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B15">
         <v>0.53320000000000001</v>
@@ -1740,7 +1743,7 @@
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B16">
         <v>1.4800000000000001E-2</v>
@@ -1757,7 +1760,7 @@
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B17">
         <v>0</v>
@@ -1774,7 +1777,7 @@
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B18">
         <v>9.9199999999999997E-2</v>
@@ -1791,7 +1794,7 @@
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B19">
         <v>0.50609999999999999</v>
@@ -1808,7 +1811,7 @@
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B20">
         <v>0.52849999999999997</v>
@@ -1825,7 +1828,7 @@
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A23" s="3" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
   </sheetData>
@@ -1843,27 +1846,27 @@
   <sheetData>
     <row r="1" spans="1:5" ht="17.399999999999999" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" s="2"/>
       <c r="B2" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="D2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="E2" s="2" t="s">
         <v>3</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="B3">
         <v>0.31759999999999999</v>
@@ -1880,7 +1883,7 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B4">
         <v>0.57640000000000002</v>
@@ -1897,7 +1900,7 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B5">
         <v>0.15340000000000001</v>
@@ -1914,7 +1917,7 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B6">
         <v>4.0300000000000002E-2</v>
@@ -1931,7 +1934,7 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B7">
         <v>9.7100000000000006E-2</v>
@@ -1948,7 +1951,7 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B8">
         <v>0.13589999999999999</v>
@@ -1965,7 +1968,7 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B9">
         <v>2.2499999999999999E-2</v>
@@ -1982,7 +1985,7 @@
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B10">
         <v>0.16270000000000001</v>
@@ -1999,7 +2002,7 @@
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B11">
         <v>0.54720000000000002</v>
@@ -2016,7 +2019,7 @@
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B12">
         <v>0.55710000000000004</v>
@@ -2033,7 +2036,7 @@
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B13">
         <v>0.96930000000000005</v>
@@ -2050,7 +2053,7 @@
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B14">
         <v>0.17150000000000001</v>
@@ -2067,7 +2070,7 @@
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B15">
         <v>3.7000000000000002E-3</v>
@@ -2084,7 +2087,7 @@
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B16">
         <v>0.9677</v>
@@ -2101,7 +2104,7 @@
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B17">
         <v>0.84899999999999998</v>
@@ -2118,7 +2121,7 @@
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B18">
         <v>0.70179999999999998</v>
@@ -2135,7 +2138,7 @@
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B19">
         <v>0.32019999999999998</v>
@@ -2152,7 +2155,7 @@
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B20">
         <v>0.30609999999999998</v>
@@ -2169,7 +2172,7 @@
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A23" s="3" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
   </sheetData>

</xml_diff>